<commit_message>
Table: keep PL's taller amikacin rows (4-5)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/IV-ATB-Renal-Adjustment_TABLE_EN+TH.xlsx
+++ b/IV-ATB-Renal-Adjustment_TABLE_EN+TH.xlsx
@@ -732,7 +732,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="56" customHeight="1">
+    <row r="4" ht="140" customHeight="1">
       <c r="A4" s="42" t="n">
         <v>1</v>
       </c>
@@ -782,7 +782,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="56" customHeight="1">
+    <row r="5" ht="112" customHeight="1">
       <c r="A5" s="32" t="n"/>
       <c r="B5" s="32" t="n"/>
       <c r="C5" s="32" t="n"/>

</xml_diff>

<commit_message>
Gentamicin: add HDEI caution note for CrCl <40
Same UpToDate sentence as amikacin (Gentamicin, Kidney Impairment, HDEI).
Table comments (rows 23-24 made taller), rules workbook and app; sw.js CACHE renal-v4.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/IV-ATB-Renal-Adjustment_TABLE_EN+TH.xlsx
+++ b/IV-ATB-Renal-Adjustment_TABLE_EN+TH.xlsx
@@ -1541,7 +1541,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="56" customHeight="1">
+    <row r="23" ht="84" customHeight="1">
       <c r="A23" s="44" t="n">
         <v>15</v>
       </c>
@@ -1586,11 +1586,12 @@
       <c r="I23" s="34" t="inlineStr">
         <is>
           <t>1. ปรับตาม Actual Body Weight (ปรับถ้า obese)
-2. ติดตามการทำงานของไตและการได้ยิน</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="56" customHeight="1">
+2. ติดตามการทำงานของไตและการได้ยิน
+3. HDEI: ใช้ด้วยความระวังเมื่อ CrCl &lt;40 แต่ยังอาจพิจารณาได้ โดยเฉพาะผู้ป่วย severe sepsis/shock หรือติดเชื้อแบคทีเรียแกรมลบดื้อยาหลายขนาน (multidrug-resistant gram-negative)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="84" customHeight="1">
       <c r="A24" s="32" t="n"/>
       <c r="B24" s="32" t="n"/>
       <c r="C24" s="32" t="n"/>

</xml_diff>